<commit_message>
updated dashboards, added statistics
</commit_message>
<xml_diff>
--- a/source.xlsx
+++ b/source.xlsx
@@ -12,6 +12,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="tasks" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="metrics" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="plans" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="dashboards" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="charts" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="chart_data" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1601,4 +1604,1086 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="35" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>columns</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>analytics</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Аналітика документів</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>⬆️ id сторінки</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Заголовок дашборду</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Кількість колонок (2 або 3)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>dashboard_id</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>type</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>color</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>order</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>analytics</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>docs_by_client</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Кількість документів з типами клієнтів</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>bar</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>#4F7CFF</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>analytics</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>docs_dynamics</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Динаміка документів за 2026</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>bar</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>#6C8AFF</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>analytics</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>docs_by_system</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Кількість документів у розрізі систем</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>bar</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>#4F7CFF</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>analytics</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>files_dynamics</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Динаміка обсягу файлів за 2026</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>bar</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>#6C8AFF</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>analytics</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>files_by_process</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Обсяг файлів за 2026 у розрізі процесів</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>bar</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>#4F7CFF</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>analytics</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>deleted_gb</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Видалено GB по місяцях</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>bar</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>#EF4444</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>⬆️ = id з dashboards</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Унікальний id графіка</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Заголовок</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>bar / line / horizontal_bar</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>HEX-колір</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>Порядок (1,2,3...)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D44"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>chart_id</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>label</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>value</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>sub</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>docs_by_client</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>ФО</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>126827084</v>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>+3.4 тис</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>docs_by_client</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>ЮО</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>3248988</v>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>+90 тис</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>docs_by_client</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>СПД</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>2260084</v>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>+59 тис</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>docs_by_client</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Самозайняті</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>14259</v>
+      </c>
+      <c r="D5" s="2" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>docs_by_client</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Банк</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>6388</v>
+      </c>
+      <c r="D6" s="2" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>docs_by_client</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Представництва ЮО</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>4369</v>
+      </c>
+      <c r="D7" s="2" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>docs_by_client</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Держ.установи</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="n">
+        <v>37</v>
+      </c>
+      <c r="D8" s="2" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>docs_dynamics</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>2026-01</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="n">
+        <v>1731828</v>
+      </c>
+      <c r="D9" s="2" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>docs_dynamics</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>2026-02</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="n">
+        <v>1785237</v>
+      </c>
+      <c r="D10" s="2" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>docs_dynamics</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="n">
+        <v>1874229</v>
+      </c>
+      <c r="D11" s="2" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>docs_by_system</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>IOS</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="n">
+        <v>980000</v>
+      </c>
+      <c r="D12" s="2" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>docs_by_system</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>CIB_SP</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="n">
+        <v>850000</v>
+      </c>
+      <c r="D13" s="2" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>docs_by_system</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Android</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="n">
+        <v>780000</v>
+      </c>
+      <c r="D14" s="2" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>docs_by_system</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>UCP</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="n">
+        <v>650000</v>
+      </c>
+      <c r="D15" s="2" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>docs_by_system</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>LKP</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="n">
+        <v>420000</v>
+      </c>
+      <c r="D16" s="2" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>docs_by_system</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>DIGITAL</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="n">
+        <v>380000</v>
+      </c>
+      <c r="D17" s="2" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>docs_by_system</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>FW</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="n">
+        <v>320000</v>
+      </c>
+      <c r="D18" s="2" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>docs_by_system</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>BWM</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="n">
+        <v>280000</v>
+      </c>
+      <c r="D19" s="2" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>docs_by_system</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>EPA</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="n">
+        <v>210000</v>
+      </c>
+      <c r="D20" s="2" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>docs_by_system</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>CLIENTBANK</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="n">
+        <v>180000</v>
+      </c>
+      <c r="D21" s="2" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>docs_by_system</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>CAMS</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="n">
+        <v>150000</v>
+      </c>
+      <c r="D22" s="2" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>docs_by_system</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>CNRP</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="n">
+        <v>120000</v>
+      </c>
+      <c r="D23" s="2" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>docs_by_system</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>SHRP</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="n">
+        <v>95000</v>
+      </c>
+      <c r="D24" s="2" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>docs_by_system</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>DHA</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="n">
+        <v>80000</v>
+      </c>
+      <c r="D25" s="2" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>docs_by_system</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>SIRIUS</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="n">
+        <v>60000</v>
+      </c>
+      <c r="D26" s="2" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>files_dynamics</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>2026-01</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="n">
+        <v>660</v>
+      </c>
+      <c r="D27" s="2" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>files_dynamics</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>2026-02</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="n">
+        <v>761</v>
+      </c>
+      <c r="D28" s="2" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>files_dynamics</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="n">
+        <v>892</v>
+      </c>
+      <c r="D29" s="2" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>files_by_process</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>Кредитування фізичних</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="n">
+        <v>1064</v>
+      </c>
+      <c r="D30" s="2" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>files_by_process</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>Кредитування юридичних</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="n">
+        <v>444</v>
+      </c>
+      <c r="D31" s="2" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>files_by_process</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>Картки фізичних</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="n">
+        <v>169</v>
+      </c>
+      <c r="D32" s="2" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>files_by_process</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>Конверсія картка</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="n">
+        <v>92</v>
+      </c>
+      <c r="D33" s="2" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>files_by_process</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>Авторизація</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="D34" s="2" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>files_by_process</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>Депозитні операції</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="n">
+        <v>66</v>
+      </c>
+      <c r="D35" s="2" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>files_by_process</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>Зарплатний проєкт</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="n">
+        <v>56</v>
+      </c>
+      <c r="D36" s="2" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>files_by_process</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>Знос бухгалтерія</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="n">
+        <v>32</v>
+      </c>
+      <c r="D37" s="2" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>files_by_process</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>Каса</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="n">
+        <v>31</v>
+      </c>
+      <c r="D38" s="2" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>files_by_process</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>Документообіг</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="D39" s="2" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>files_by_process</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>Валютні операції</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="D40" s="2" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>deleted_gb</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>Січ.26</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="n">
+        <v>823</v>
+      </c>
+      <c r="D41" s="2" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>deleted_gb</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>Лют.26</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="n">
+        <v>557</v>
+      </c>
+      <c r="D42" s="2" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>deleted_gb</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>Бер.26</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="n">
+        <v>223</v>
+      </c>
+      <c r="D43" s="2" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="3" t="inlineStr">
+        <is>
+          <t>⬆️ = id з charts</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>Підпис (вісь X)</t>
+        </is>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>Значення (число)</t>
+        </is>
+      </c>
+      <c r="D44" s="3" t="inlineStr">
+        <is>
+          <t>Додатковий текст (необов'язково)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>